<commit_message>
Add relationship-check skill and People table
Port of /enrich stale: tier cadences, last-contact refresh from real
two-way interactions, a personal reason to reach out, and
draft/track/snooze actions. Schema 0.3.0 adds the People table with
linter checks and eval fixtures.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QAFSVUxnFJr1GcBNuVRsg1
</commit_message>
<xml_diff>
--- a/m365/workbook/ChiefOfStaff.xlsx
+++ b/m365/workbook/ChiefOfStaff.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goals" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedback" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -289,6 +290,25 @@
     <tableColumn id="7" name="Theme"/>
     <tableColumn id="8" name="Applied"/>
     <tableColumn id="9" name="ResultingChange"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="People" displayName="People" ref="A1:J2" headerRowCount="1">
+  <autoFilter ref="A1:J2"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Email"/>
+    <tableColumn id="2" name="Name"/>
+    <tableColumn id="3" name="Tier"/>
+    <tableColumn id="4" name="Role"/>
+    <tableColumn id="5" name="CadenceDays"/>
+    <tableColumn id="6" name="LastContact"/>
+    <tableColumn id="7" name="LastChannel"/>
+    <tableColumn id="8" name="Notes"/>
+    <tableColumn id="9" name="NextTouch"/>
+    <tableColumn id="10" name="Updated"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -1337,7 +1357,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CadenceDays</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LastContact</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>LastChannel</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>NextTouch</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"email,teams,meeting,call,in_person"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1357,7 +1478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema v0.2.0 - generated from m365/schema/workbook.yaml. Edit the schema, not this sheet.</t>
+          <t>Schema v0.3.0 - generated from m365/schema/workbook.yaml. Edit the schema, not this sheet.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -2279,6 +2400,145 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>People  (sheet: People, key: Email)</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr"/>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>Relationships worth keeping warm. Tier sets the check-in cadence (1 = 14 days, 2 = 30, 3 = 60).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Email</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>key; lowercase</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Name</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Tier</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>1 inner circle · 2 active network · 3 extended</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Role</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>role and company</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CadenceDays</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>optional override of the tier cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    LastContact</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>latest two-way interaction found</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    LastChannel</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>email, teams, meeting, call, in_person</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Notes</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>one per line, dated: 'Training for a marathon (added 2026-10-29)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    NextTouch</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>suggested reason to reach out, refreshed by relationship-check</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Updated</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>